<commit_message>
Improve CSV/XLSX parsing and dataset handling
Enhance frontend parsing/export and preserve full dataset while improving Excel handling on the backend. Frontend: add robust CSV line parser (handles quoted values and escaped quotes), proper CSV escaping and output filename, more resilient XLSX parsing that skips empty leading rows, maps columns by header indices, and builds consistent data objects; use payload.dataset when available to preserve full dataset in multiple flows; tweak user-facing error messages. Backend: pass engine="calamine" to read_excel_clean in ml_service and add an engine parameter to utils.read_excel_clean so pandas.read_excel can use the provided engine. Add python-calamine to installs and include updated sample Excel files.
</commit_message>
<xml_diff>
--- a/Input/Project-Management-Sample-Data.xlsx
+++ b/Input/Project-Management-Sample-Data.xlsx
@@ -2,15 +2,15 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
-  <workbookPr/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\cs\GP\AutoPrepAI\AutoPrepAI\Input\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\zinab\Documents\GitHub\AutoPrepAI\Input\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6A3A2A51-2B40-4889-A67B-288861DF1AD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1909FB23-EB5B-4679-AA0A-61C2F023AE1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{CE120CA2-B4E2-4FC9-9B81-FB00098FDFE6}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" xr2:uid="{CE120CA2-B4E2-4FC9-9B81-FB00098FDFE6}"/>
   </bookViews>
   <sheets>
     <sheet name="Project Management Data" sheetId="2" r:id="rId1"/>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="102">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="129" uniqueCount="100">
   <si>
     <t>Project Name</t>
   </si>
@@ -325,19 +325,13 @@
   </si>
   <si>
     <t>Oscar</t>
-  </si>
-  <si>
-    <t>Excel Sample Data</t>
-  </si>
-  <si>
-    <t>Project Management Data</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -790,18 +784,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3FC7BEC1-BD91-4F4F-8985-8014BC582418}">
   <dimension ref="A1:G47"/>
-  <sheetFormatPr defaultColWidth="9.125" defaultRowHeight="18" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="9.109375" defaultRowHeight="18" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="15.5" style="1" customWidth="1"/>
+    <col min="1" max="1" width="15.44140625" style="1" customWidth="1"/>
     <col min="2" max="2" width="25" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="4" width="13.5" style="1" customWidth="1"/>
-    <col min="5" max="5" width="15.5" style="1" customWidth="1"/>
-    <col min="6" max="6" width="16.5" style="1" customWidth="1"/>
+    <col min="3" max="4" width="13.44140625" style="1" customWidth="1"/>
+    <col min="5" max="5" width="15.44140625" style="1" customWidth="1"/>
+    <col min="6" max="6" width="16.44140625" style="1" customWidth="1"/>
     <col min="7" max="7" width="17" style="1" customWidth="1"/>
-    <col min="8" max="16384" width="9.125" style="1"/>
+    <col min="8" max="16384" width="9.109375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="18" customHeight="1">
+    <row r="1" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A1" s="6"/>
       <c r="B1" s="6"/>
       <c r="C1" s="4"/>
@@ -810,18 +804,16 @@
       <c r="F1" s="4"/>
       <c r="G1" s="4"/>
     </row>
-    <row r="2" spans="1:7" ht="18" customHeight="1" thickBot="1">
+    <row r="2" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="4"/>
-      <c r="B2" s="7" t="s">
-        <v>100</v>
-      </c>
+      <c r="B2" s="7"/>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
       <c r="E2" s="7"/>
       <c r="F2" s="7"/>
       <c r="G2" s="7"/>
     </row>
-    <row r="3" spans="1:7" ht="18" customHeight="1">
+    <row r="3" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6"/>
       <c r="B3" s="6"/>
       <c r="C3" s="4"/>
@@ -830,18 +822,16 @@
       <c r="F3" s="4"/>
       <c r="G3" s="4"/>
     </row>
-    <row r="4" spans="1:7" ht="18" customHeight="1" thickBot="1">
+    <row r="4" spans="1:7" ht="18" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A4" s="4"/>
-      <c r="B4" s="8" t="s">
-        <v>101</v>
-      </c>
+      <c r="B4" s="8"/>
       <c r="C4" s="8"/>
       <c r="D4" s="8"/>
       <c r="E4" s="8"/>
       <c r="F4" s="8"/>
       <c r="G4" s="8"/>
     </row>
-    <row r="5" spans="1:7" ht="18" customHeight="1">
+    <row r="5" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6"/>
       <c r="B5" s="6"/>
       <c r="C5" s="4"/>
@@ -850,7 +840,7 @@
       <c r="F5" s="4"/>
       <c r="G5" s="4"/>
     </row>
-    <row r="6" spans="1:7" ht="18" customHeight="1">
+    <row r="6" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="4"/>
       <c r="B6" s="5" t="s">
         <v>0</v>
@@ -871,7 +861,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="18" customHeight="1">
+    <row r="7" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="4"/>
       <c r="B7" s="2" t="s">
         <v>6</v>
@@ -892,7 +882,7 @@
         <v>45305</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="18" customHeight="1">
+    <row r="8" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A8" s="4"/>
       <c r="B8" s="2" t="s">
         <v>6</v>
@@ -913,7 +903,7 @@
         <v>45319</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="18" customHeight="1">
+    <row r="9" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="4"/>
       <c r="B9" s="2" t="s">
         <v>6</v>
@@ -934,7 +924,7 @@
         <v>45341</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="18" customHeight="1">
+    <row r="10" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="4"/>
       <c r="B10" s="2" t="s">
         <v>6</v>
@@ -955,7 +945,7 @@
         <v>45365</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="18" customHeight="1">
+    <row r="11" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="4"/>
       <c r="B11" s="2" t="s">
         <v>15</v>
@@ -976,7 +966,7 @@
         <v>45311</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="18" customHeight="1">
+    <row r="12" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="4"/>
       <c r="B12" s="2" t="s">
         <v>15</v>
@@ -997,7 +987,7 @@
         <v>45321</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="18" customHeight="1">
+    <row r="13" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="4"/>
       <c r="B13" s="2" t="s">
         <v>15</v>
@@ -1018,7 +1008,7 @@
         <v>45351</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="18" customHeight="1">
+    <row r="14" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="4"/>
       <c r="B14" s="2" t="s">
         <v>22</v>
@@ -1039,7 +1029,7 @@
         <v>45345</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="18" customHeight="1">
+    <row r="15" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="4"/>
       <c r="B15" s="2" t="s">
         <v>22</v>
@@ -1060,7 +1050,7 @@
         <v>45371</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="18" customHeight="1">
+    <row r="16" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="4"/>
       <c r="B16" s="2" t="s">
         <v>22</v>
@@ -1081,7 +1071,7 @@
         <v>45402</v>
       </c>
     </row>
-    <row r="17" spans="1:7" ht="18" customHeight="1">
+    <row r="17" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A17" s="4"/>
       <c r="B17" s="2" t="s">
         <v>29</v>
@@ -1102,7 +1092,7 @@
         <v>45346</v>
       </c>
     </row>
-    <row r="18" spans="1:7" ht="18" customHeight="1">
+    <row r="18" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="4"/>
       <c r="B18" s="2" t="s">
         <v>29</v>
@@ -1123,7 +1113,7 @@
         <v>45331</v>
       </c>
     </row>
-    <row r="19" spans="1:7" ht="18" customHeight="1">
+    <row r="19" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A19" s="4"/>
       <c r="B19" s="2" t="s">
         <v>29</v>
@@ -1144,7 +1134,7 @@
         <v>45395</v>
       </c>
     </row>
-    <row r="20" spans="1:7" ht="18" customHeight="1">
+    <row r="20" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="4"/>
       <c r="B20" s="2" t="s">
         <v>35</v>
@@ -1165,7 +1155,7 @@
         <v>45316</v>
       </c>
     </row>
-    <row r="21" spans="1:7" ht="18" customHeight="1">
+    <row r="21" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="4"/>
       <c r="B21" s="2" t="s">
         <v>35</v>
@@ -1186,7 +1176,7 @@
         <v>45349</v>
       </c>
     </row>
-    <row r="22" spans="1:7" ht="18" customHeight="1">
+    <row r="22" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="4"/>
       <c r="B22" s="2" t="s">
         <v>35</v>
@@ -1207,7 +1197,7 @@
         <v>45377</v>
       </c>
     </row>
-    <row r="23" spans="1:7" ht="18" customHeight="1">
+    <row r="23" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="4"/>
       <c r="B23" s="2" t="s">
         <v>42</v>
@@ -1228,7 +1218,7 @@
         <v>45329</v>
       </c>
     </row>
-    <row r="24" spans="1:7" ht="18" customHeight="1">
+    <row r="24" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="4"/>
       <c r="B24" s="2" t="s">
         <v>42</v>
@@ -1249,7 +1239,7 @@
         <v>45364</v>
       </c>
     </row>
-    <row r="25" spans="1:7" ht="18" customHeight="1">
+    <row r="25" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="4"/>
       <c r="B25" s="2" t="s">
         <v>42</v>
@@ -1270,7 +1260,7 @@
         <v>45395</v>
       </c>
     </row>
-    <row r="26" spans="1:7" ht="18" customHeight="1">
+    <row r="26" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="4"/>
       <c r="B26" s="2" t="s">
         <v>49</v>
@@ -1291,7 +1281,7 @@
         <v>45341</v>
       </c>
     </row>
-    <row r="27" spans="1:7" ht="18" customHeight="1">
+    <row r="27" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="4"/>
       <c r="B27" s="2" t="s">
         <v>49</v>
@@ -1312,7 +1302,7 @@
         <v>45366</v>
       </c>
     </row>
-    <row r="28" spans="1:7" ht="18" customHeight="1">
+    <row r="28" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="4"/>
       <c r="B28" s="2" t="s">
         <v>49</v>
@@ -1333,7 +1323,7 @@
         <v>45387</v>
       </c>
     </row>
-    <row r="29" spans="1:7" ht="18" customHeight="1">
+    <row r="29" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="4"/>
       <c r="B29" s="2" t="s">
         <v>56</v>
@@ -1354,7 +1344,7 @@
         <v>45354</v>
       </c>
     </row>
-    <row r="30" spans="1:7" ht="18" customHeight="1">
+    <row r="30" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="4"/>
       <c r="B30" s="2" t="s">
         <v>56</v>
@@ -1375,7 +1365,7 @@
         <v>45317</v>
       </c>
     </row>
-    <row r="31" spans="1:7" ht="18" customHeight="1">
+    <row r="31" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="4"/>
       <c r="B31" s="2" t="s">
         <v>56</v>
@@ -1396,7 +1386,7 @@
         <v>45360</v>
       </c>
     </row>
-    <row r="32" spans="1:7" ht="18" customHeight="1">
+    <row r="32" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="4"/>
       <c r="B32" s="2" t="s">
         <v>63</v>
@@ -1417,7 +1407,7 @@
         <v>45317</v>
       </c>
     </row>
-    <row r="33" spans="1:7" ht="18" customHeight="1">
+    <row r="33" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="4"/>
       <c r="B33" s="2" t="s">
         <v>63</v>
@@ -1438,7 +1428,7 @@
         <v>45349</v>
       </c>
     </row>
-    <row r="34" spans="1:7" ht="18" customHeight="1">
+    <row r="34" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="4"/>
       <c r="B34" s="2" t="s">
         <v>63</v>
@@ -1459,7 +1449,7 @@
         <v>45375</v>
       </c>
     </row>
-    <row r="35" spans="1:7" ht="18" customHeight="1">
+    <row r="35" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="4"/>
       <c r="B35" s="2" t="s">
         <v>70</v>
@@ -1480,7 +1470,7 @@
         <v>45324</v>
       </c>
     </row>
-    <row r="36" spans="1:7" ht="18" customHeight="1">
+    <row r="36" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="4"/>
       <c r="B36" s="2" t="s">
         <v>70</v>
@@ -1501,7 +1491,7 @@
         <v>45350</v>
       </c>
     </row>
-    <row r="37" spans="1:7" ht="18" customHeight="1">
+    <row r="37" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="4"/>
       <c r="B37" s="2" t="s">
         <v>70</v>
@@ -1522,7 +1512,7 @@
         <v>45371</v>
       </c>
     </row>
-    <row r="38" spans="1:7" ht="18" customHeight="1">
+    <row r="38" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="4"/>
       <c r="B38" s="2" t="s">
         <v>77</v>
@@ -1543,7 +1533,7 @@
         <v>45328</v>
       </c>
     </row>
-    <row r="39" spans="1:7" ht="18" customHeight="1">
+    <row r="39" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="4"/>
       <c r="B39" s="2" t="s">
         <v>77</v>
@@ -1564,7 +1554,7 @@
         <v>45356</v>
       </c>
     </row>
-    <row r="40" spans="1:7" ht="18" customHeight="1">
+    <row r="40" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="4"/>
       <c r="B40" s="2" t="s">
         <v>77</v>
@@ -1585,7 +1575,7 @@
         <v>45382</v>
       </c>
     </row>
-    <row r="41" spans="1:7" ht="18" customHeight="1">
+    <row r="41" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="4"/>
       <c r="B41" s="2" t="s">
         <v>83</v>
@@ -1606,7 +1596,7 @@
         <v>45322</v>
       </c>
     </row>
-    <row r="42" spans="1:7" ht="18" customHeight="1">
+    <row r="42" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="4"/>
       <c r="B42" s="2" t="s">
         <v>83</v>
@@ -1627,7 +1617,7 @@
         <v>45349</v>
       </c>
     </row>
-    <row r="43" spans="1:7" ht="18" customHeight="1">
+    <row r="43" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="4"/>
       <c r="B43" s="2" t="s">
         <v>83</v>
@@ -1648,7 +1638,7 @@
         <v>45372</v>
       </c>
     </row>
-    <row r="44" spans="1:7" ht="18" customHeight="1">
+    <row r="44" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="4"/>
       <c r="B44" s="2" t="s">
         <v>90</v>
@@ -1669,7 +1659,7 @@
         <v>45319</v>
       </c>
     </row>
-    <row r="45" spans="1:7" ht="18" customHeight="1">
+    <row r="45" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="4"/>
       <c r="B45" s="2" t="s">
         <v>90</v>
@@ -1690,7 +1680,7 @@
         <v>45345</v>
       </c>
     </row>
-    <row r="46" spans="1:7" ht="18" customHeight="1">
+    <row r="46" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="4"/>
       <c r="B46" s="2" t="s">
         <v>90</v>
@@ -1711,7 +1701,7 @@
         <v>45381</v>
       </c>
     </row>
-    <row r="47" spans="1:7" ht="18" customHeight="1">
+    <row r="47" spans="1:7" ht="18" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="4"/>
       <c r="B47" s="2" t="s">
         <v>97</v>

</xml_diff>